<commit_message>
Bai 29 Data provider (chạy tuần tự)
</commit_message>
<xml_diff>
--- a/src/test/resources/DataTest/Customers.xlsx
+++ b/src/test/resources/DataTest/Customers.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18650" windowHeight="6930" activeTab="1"/>
+    <workbookView windowWidth="18650" windowHeight="6930"/>
   </bookViews>
   <sheets>
     <sheet name="AddCustomer" sheetId="1" r:id="rId1"/>
@@ -130,10 +130,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -158,16 +158,22 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -188,13 +194,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="3"/>
@@ -221,23 +220,29 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -251,6 +256,7 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -259,36 +265,30 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -303,6 +303,54 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -315,7 +363,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -333,7 +405,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -345,19 +435,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -369,31 +447,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -405,13 +465,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -423,67 +477,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -497,35 +497,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -554,13 +530,41 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -580,32 +584,28 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
+      <left/>
+      <right/>
       <top style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color theme="4"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -615,130 +615,130 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="24" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>

<commit_message>
refactor input add customer, demo data provider add customer
</commit_message>
<xml_diff>
--- a/src/test/resources/DataTest/Customers.xlsx
+++ b/src/test/resources/DataTest/Customers.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="39">
   <si>
     <t>Company</t>
   </si>
@@ -53,7 +53,13 @@
     <t>Country</t>
   </si>
   <si>
-    <t>T_Test13012026</t>
+    <t>T_Test0_17012026</t>
+  </si>
+  <si>
+    <t>T_Test1_17012026</t>
+  </si>
+  <si>
+    <t>10</t>
   </si>
   <si>
     <t>0123456789</t>
@@ -65,7 +71,7 @@
     <t>Gold</t>
   </si>
   <si>
-    <t>USD$</t>
+    <t>USD</t>
   </si>
   <si>
     <t>English</t>
@@ -80,10 +86,13 @@
     <t>Quan 11</t>
   </si>
   <si>
+    <t>123</t>
+  </si>
+  <si>
     <t>United States</t>
   </si>
   <si>
-    <t>T_Test2_130126</t>
+    <t>T_Test2_170126</t>
   </si>
   <si>
     <t>VAT123</t>
@@ -95,13 +104,13 @@
     <t>google.com</t>
   </si>
   <si>
-    <t>T_Test3_130126</t>
-  </si>
-  <si>
-    <t>T_Test4_130126</t>
-  </si>
-  <si>
-    <t>T_Test6_130126</t>
+    <t>T_Test3_170126</t>
+  </si>
+  <si>
+    <t>T_Test4_170126</t>
+  </si>
+  <si>
+    <t>T_Test6_170126</t>
   </si>
   <si>
     <t>FirstName</t>
@@ -116,13 +125,13 @@
     <t>Password</t>
   </si>
   <si>
-    <t>binh1</t>
-  </si>
-  <si>
-    <t>an1</t>
-  </si>
-  <si>
-    <t>binhan1@alert.com</t>
+    <t>binh2</t>
+  </si>
+  <si>
+    <t>an2</t>
+  </si>
+  <si>
+    <t>binhan2@alert.com</t>
   </si>
 </sst>
 </file>
@@ -130,10 +139,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -159,21 +168,21 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -202,6 +211,90 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="18"/>
       <color theme="3"/>
@@ -209,90 +302,6 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -303,18 +312,168 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -327,163 +486,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -500,8 +509,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -510,7 +519,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -545,30 +554,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -594,18 +579,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -615,130 +624,130 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="24" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1066,16 +1075,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="5"/>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="6"/>
   <cols>
-    <col min="1" max="1" width="15.6363636363636" customWidth="1"/>
+    <col min="1" max="1" width="20.3636363636364" customWidth="1"/>
     <col min="2" max="2" width="12.2727272727273" customWidth="1"/>
     <col min="3" max="3" width="14.5454545454545" customWidth="1"/>
     <col min="4" max="4" width="14.0909090909091" customWidth="1"/>
     <col min="7" max="7" width="16.9090909090909" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="12.0909090909091" customWidth="1"/>
+    <col min="12" max="12" width="15.5454545454545" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -1120,157 +1130,163 @@
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2">
-        <v>10</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2">
-        <v>123</v>
-      </c>
-      <c r="L2" t="s">
-        <v>21</v>
-      </c>
+      <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" t="s">
+      <c r="K3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="L3" t="s">
         <v>24</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
         <v>25</v>
       </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s">
         <v>17</v>
       </c>
-      <c r="H3" t="s">
+      <c r="F4" t="s">
         <v>18</v>
       </c>
-      <c r="I3" t="s">
+      <c r="G4" t="s">
         <v>19</v>
       </c>
-      <c r="J3" t="s">
+      <c r="H4" t="s">
         <v>20</v>
       </c>
-      <c r="K3">
-        <v>123</v>
-      </c>
-      <c r="L3" t="s">
+      <c r="I4" t="s">
         <v>21</v>
       </c>
+      <c r="J4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" t="s">
-        <v>19</v>
-      </c>
-      <c r="J5" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5">
-        <v>123</v>
-      </c>
-      <c r="L5" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" t="s">
         <v>28</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="L6" t="s">
         <v>24</v>
       </c>
-      <c r="D6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" t="s">
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" t="s">
         <v>17</v>
       </c>
-      <c r="H6" t="s">
+      <c r="F7" t="s">
         <v>18</v>
       </c>
-      <c r="I6" t="s">
+      <c r="G7" t="s">
         <v>19</v>
       </c>
-      <c r="J6" t="s">
+      <c r="H7" t="s">
         <v>20</v>
       </c>
-      <c r="K6">
-        <v>123</v>
-      </c>
-      <c r="L6" t="s">
+      <c r="I7" t="s">
         <v>21</v>
+      </c>
+      <c r="J7" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L7" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1293,27 +1309,27 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D2">
         <v>123456</v>
@@ -1321,7 +1337,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="binhan1@alert.com" tooltip="mailto:binhan1@alert.com"/>
+    <hyperlink ref="C2" r:id="rId1" display="binhan2@alert.com" tooltip="mailto:binhan2@alert.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>